<commit_message>
remove no document from bulk
</commit_message>
<xml_diff>
--- a/storage/app/public/template/Template Asset Bulk.xlsx
+++ b/storage/app/public/template/Template Asset Bulk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\lrt-demo1\storage\app\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A1D800-88BA-4AD0-9316-065DF4E01386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{275C6ACE-EEF2-4319-AEFF-6FB08D937272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
   <si>
     <t>Asset Number Internal</t>
   </si>
@@ -76,9 +76,6 @@
     <t>PPA-2006-00332</t>
   </si>
   <si>
-    <t>JB-2007-00277 : FAACQ</t>
-  </si>
-  <si>
     <t>MPS2007000002</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
   </si>
   <si>
     <t>Nota Referensi</t>
-  </si>
-  <si>
-    <t>No Document</t>
   </si>
   <si>
     <t>A1100000001</t>
@@ -519,34 +513,33 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="26.28515625" customWidth="1"/>
     <col min="7" max="7" width="26.140625" customWidth="1"/>
     <col min="8" max="8" width="37.85546875" customWidth="1"/>
     <col min="9" max="29" width="26.28515625" customWidth="1"/>
-    <col min="30" max="30" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>17</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>0</v>
@@ -570,66 +563,63 @@
         <v>6</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="P1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="T1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="U1" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>9</v>
       </c>
       <c r="W1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="X1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="X1" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="Y1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="4" t="s">
+      <c r="AA1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AA1" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="AB1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AC1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="AD1" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
-        <v>35</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D2" s="11">
         <v>1100</v>
@@ -640,7 +630,7 @@
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="6">
@@ -650,13 +640,13 @@
         <v>44013</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M2" s="5">
         <v>1</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O2" s="7">
         <v>82500000</v>
@@ -686,7 +676,7 @@
         <v>0</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Y2" s="5" t="s">
         <v>12</v>
@@ -701,42 +691,39 @@
       <c r="AC2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="AD2" s="3" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="3" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D3" s="11">
         <v>1101</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M3" s="5">
         <v>1</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O3" s="7">
         <v>154550000</v>
@@ -760,7 +747,7 @@
         <v>0</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Y3" s="5" t="s">
         <v>12</v>
@@ -774,9 +761,6 @@
       <c r="AB3" s="5"/>
       <c r="AC3" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="AD3" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add notes to bulk excel
</commit_message>
<xml_diff>
--- a/storage/app/public/template/Template Asset Bulk.xlsx
+++ b/storage/app/public/template/Template Asset Bulk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\lrt-demo1\storage\app\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{275C6ACE-EEF2-4319-AEFF-6FB08D937272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D2D351-8391-4670-81AC-131E6DB3730D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>Asset Number Internal</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t>00</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
@@ -227,7 +230,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -250,11 +253,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -262,9 +293,6 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -295,6 +323,16 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,106 +551,110 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="26.28515625" customWidth="1"/>
     <col min="7" max="7" width="26.140625" customWidth="1"/>
     <col min="8" max="8" width="37.85546875" customWidth="1"/>
     <col min="9" max="29" width="26.28515625" customWidth="1"/>
+    <col min="30" max="30" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="V1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="W1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="X1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="Z1" s="4" t="s">
+      <c r="Z1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AA1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AB1" s="4" t="s">
+      <c r="AB1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AC1" s="4" t="s">
+      <c r="AC1" s="13" t="s">
         <v>32</v>
       </c>
+      <c r="AD1" s="15" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
         <v>33</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -621,79 +663,80 @@
       <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="10">
         <v>1100</v>
       </c>
-      <c r="E2" s="5"/>
+      <c r="E2" s="4"/>
       <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="10" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="5"/>
-      <c r="J2" s="6">
+      <c r="I2" s="4"/>
+      <c r="J2" s="5">
         <v>44013</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="5">
         <v>44013</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="4">
         <v>1</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="7">
+      <c r="O2" s="6">
         <v>82500000</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="Q2" s="8">
+      <c r="Q2" s="7">
         <v>82500001</v>
       </c>
-      <c r="R2" s="5">
+      <c r="R2" s="4">
         <v>48</v>
       </c>
-      <c r="S2" s="9">
+      <c r="S2" s="8">
         <v>-72187500</v>
       </c>
-      <c r="T2" s="9">
+      <c r="T2" s="8">
         <v>-1718750</v>
       </c>
-      <c r="U2" s="9">
+      <c r="U2" s="8">
         <v>-10312500</v>
       </c>
-      <c r="V2" s="9">
+      <c r="V2" s="8">
         <v>-82500000</v>
       </c>
-      <c r="W2" s="5">
+      <c r="W2" s="4">
         <v>0</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="X2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="5" t="s">
+      <c r="Y2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="Z2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="AA2" s="5" t="s">
+      <c r="AA2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="AB2" s="5"/>
-      <c r="AC2" s="3" t="s">
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="14" t="s">
         <v>13</v>
       </c>
+      <c r="AD2" s="16"/>
     </row>
-    <row r="3" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
         <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -702,66 +745,67 @@
       <c r="C3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="10">
         <v>1101</v>
       </c>
-      <c r="E3" s="5"/>
+      <c r="E3" s="4"/>
       <c r="F3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="10" t="s">
+      <c r="G3" s="4"/>
+      <c r="H3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="5"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="5" t="s">
+      <c r="I3" s="4"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3" s="4">
         <v>1</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="O3" s="7">
+      <c r="O3" s="6">
         <v>154550000</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="P3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="5">
+      <c r="Q3" s="7"/>
+      <c r="R3" s="4">
         <v>48</v>
       </c>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9">
+      <c r="S3" s="8"/>
+      <c r="T3" s="8">
         <v>0</v>
       </c>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9">
+      <c r="U3" s="8"/>
+      <c r="V3" s="8">
         <v>0</v>
       </c>
-      <c r="W3" s="5">
+      <c r="W3" s="4">
         <v>0</v>
       </c>
-      <c r="X3" s="5" t="s">
+      <c r="X3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="Y3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="Z3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="AA3" s="5" t="s">
+      <c r="AA3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="AB3" s="5"/>
-      <c r="AC3" s="3" t="s">
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="14" t="s">
         <v>13</v>
       </c>
+      <c r="AD3" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixing bulk upload and acquisition insert rules
</commit_message>
<xml_diff>
--- a/storage/app/public/template/Template Asset Bulk.xlsx
+++ b/storage/app/public/template/Template Asset Bulk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\lrt-demo1\storage\app\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D2D351-8391-4670-81AC-131E6DB3730D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303793CE-9B1C-48AD-845A-867057F9A565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="40">
   <si>
     <t>Asset Number Internal</t>
   </si>
@@ -58,12 +58,6 @@
     <t>Pajak</t>
   </si>
   <si>
-    <t>Begining</t>
-  </si>
-  <si>
-    <t>Ending Balance</t>
-  </si>
-  <si>
     <t>MPS2007000001</t>
   </si>
   <si>
@@ -95,15 +89,6 @@
   </si>
   <si>
     <t>KG</t>
-  </si>
-  <si>
-    <t>Addition Month</t>
-  </si>
-  <si>
-    <t>Total Adition</t>
-  </si>
-  <si>
-    <t>Net Book value</t>
   </si>
   <si>
     <t>Asset Status</t>
@@ -285,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -306,9 +291,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -551,34 +533,34 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="26.28515625" customWidth="1"/>
     <col min="7" max="7" width="26.140625" customWidth="1"/>
     <col min="8" max="8" width="37.85546875" customWidth="1"/>
-    <col min="9" max="29" width="26.28515625" customWidth="1"/>
-    <col min="30" max="30" width="34.7109375" customWidth="1"/>
+    <col min="9" max="24" width="26.28515625" customWidth="1"/>
+    <col min="25" max="25" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>36</v>
+        <v>33</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>0</v>
@@ -602,77 +584,62 @@
         <v>6</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Y1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Y1" s="14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AA1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC1" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD1" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
-        <v>33</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="10">
+        <v>36</v>
+      </c>
+      <c r="D2" s="9">
         <v>1100</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G2" s="4"/>
-      <c r="H2" s="9" t="s">
-        <v>18</v>
+      <c r="H2" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="5">
@@ -682,19 +649,19 @@
         <v>44013</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M2" s="4">
         <v>1</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O2" s="6">
         <v>82500000</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q2" s="7">
         <v>82500001</v>
@@ -702,110 +669,84 @@
       <c r="R2" s="4">
         <v>48</v>
       </c>
-      <c r="S2" s="8">
-        <v>-72187500</v>
-      </c>
-      <c r="T2" s="8">
-        <v>-1718750</v>
-      </c>
-      <c r="U2" s="8">
-        <v>-10312500</v>
-      </c>
-      <c r="V2" s="8">
-        <v>-82500000</v>
-      </c>
-      <c r="W2" s="4">
-        <v>0</v>
-      </c>
-      <c r="X2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="AD2" s="16"/>
+      <c r="S2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="W2" s="4"/>
+      <c r="X2" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y2" s="15"/>
     </row>
-    <row r="3" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
-        <v>34</v>
+    <row r="3" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>29</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" s="10">
+        <v>36</v>
+      </c>
+      <c r="D3" s="9">
         <v>1101</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="4"/>
-      <c r="H3" s="9" t="s">
-        <v>19</v>
+      <c r="H3" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M3" s="4">
         <v>1</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O3" s="6">
         <v>154550000</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q3" s="7"/>
       <c r="R3" s="4">
         <v>48</v>
       </c>
-      <c r="S3" s="8"/>
-      <c r="T3" s="8">
-        <v>0</v>
-      </c>
-      <c r="U3" s="8"/>
-      <c r="V3" s="8">
-        <v>0</v>
-      </c>
-      <c r="W3" s="4">
-        <v>0</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB3" s="4"/>
-      <c r="AC3" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="AD3" s="16"/>
+      <c r="S3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="W3" s="4"/>
+      <c r="X3" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y3" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>